<commit_message>
fix(db): agregar columna tipo y session_id a conciliacion_lineas
La columna tipo (cargo/abono) nunca fue migrada a la base de datos local.
Causa: 0 transacciones guardadas en todos los bancos a pesar de que el
parser leía los datos correctamente.

- Nueva migración: add_tipo_session_to_conciliacion_lineas
- tipo: string nullable default abono
- session_id: string nullable (si no existe)
</commit_message>
<xml_diff>
--- a/Nueva carpeta/BANESCO.xlsx
+++ b/Nueva carpeta/BANESCO.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\freyg\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\freyg\Downloads\laravel_app\Nueva carpeta\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17985" windowHeight="9165"/>
   </bookViews>
   <sheets>
     <sheet name="J501653879 (11)" sheetId="1" r:id="rId1"/>

</xml_diff>